<commit_message>
added 2 new columns and make UI professional
</commit_message>
<xml_diff>
--- a/public/sample/AppMappingTemplate.xlsx
+++ b/public/sample/AppMappingTemplate.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vikrantkadam/studyProject/SmartExcelJsonMapper/Client Excel Field Mapper Files/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vikrantkadam/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DBEF81D-39AB-F84C-BAE3-84D82A987903}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB717F05-D949-324F-8AE4-80B8E0FC4CB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17200" xr2:uid="{9012A801-4D30-9C46-97FB-7EB8B5E3B893}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17180" xr2:uid="{9012A801-4D30-9C46-97FB-7EB8B5E3B893}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="31">
   <si>
     <t>AppField</t>
   </si>
@@ -114,13 +114,28 @@
   </si>
   <si>
     <t>Customer</t>
+  </si>
+  <si>
+    <t>Required</t>
+  </si>
+  <si>
+    <t>Max Length</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>NA</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -142,6 +157,19 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Helvetica"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Helvetica"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -179,12 +207,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -519,165 +552,314 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA83E3A0-B305-154A-BA77-56A2878239DA}">
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="23" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="27.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1"/>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A2" s="3" t="s">
+      <c r="C1" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="4"/>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A3" s="3" t="s">
+      <c r="B2" s="3"/>
+      <c r="C2" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" s="5">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="4"/>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" s="3" t="s">
+      <c r="B3" s="3"/>
+      <c r="C3" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D3" s="5">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="4"/>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5" s="3" t="s">
+      <c r="B4" s="3"/>
+      <c r="C4" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D4" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="3"/>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A6" s="3" t="s">
+      <c r="B5" s="2"/>
+      <c r="C5" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" s="5">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="3"/>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A7" s="3" t="s">
+      <c r="B6" s="2"/>
+      <c r="C6" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D6" s="5">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="3"/>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A8" s="3" t="s">
+      <c r="B7" s="2"/>
+      <c r="C7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D7" s="5">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="4"/>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A9" s="3" t="s">
+      <c r="B8" s="3"/>
+      <c r="C8" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D8" s="5">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="3"/>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A10" s="3" t="s">
+      <c r="B9" s="2"/>
+      <c r="C9" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D9" s="5">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A10" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="4"/>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A11" s="3" t="s">
+      <c r="B10" s="3"/>
+      <c r="C10" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D10" s="5">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A11" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="4"/>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A12" s="3" t="s">
+      <c r="B11" s="3"/>
+      <c r="C11" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="3"/>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A13" s="3" t="s">
+      <c r="B12" s="2"/>
+      <c r="C12" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D12" s="5">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A13" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B13" s="3"/>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A14" s="3" t="s">
+      <c r="B13" s="2"/>
+      <c r="C13" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D13" s="5">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A14" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B14" s="3"/>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A15" s="3" t="s">
+      <c r="B14" s="2"/>
+      <c r="C14" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D14" s="5">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A15" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B15" s="3"/>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A16" s="3" t="s">
+      <c r="B15" s="2"/>
+      <c r="C15" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A16" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B16" s="3"/>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A17" s="3" t="s">
+      <c r="B16" s="2"/>
+      <c r="C16" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D16" s="5">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A17" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B17" s="4"/>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A18" s="3" t="s">
+      <c r="B17" s="3"/>
+      <c r="C17" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D17" s="5">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A18" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B18" s="4"/>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A19" s="3" t="s">
+      <c r="B18" s="3"/>
+      <c r="C18" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D18" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A19" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B19" s="3"/>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A20" s="3" t="s">
+      <c r="B19" s="2"/>
+      <c r="C19" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D19" s="5">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A20" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B20" s="3"/>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A21" s="3" t="s">
+      <c r="B20" s="2"/>
+      <c r="C20" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A21" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B21" s="3"/>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A22" s="3" t="s">
+      <c r="B21" s="2"/>
+      <c r="C21" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A22" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B22" s="3"/>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A23" s="3" t="s">
+      <c r="B22" s="2"/>
+      <c r="C22" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A23" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B23" s="3"/>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A24" s="3" t="s">
+      <c r="B23" s="2"/>
+      <c r="C23" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D23" s="5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A24" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B24" s="3"/>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A25" s="3" t="s">
+      <c r="B24" s="2"/>
+      <c r="C24" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A25" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B25" s="3"/>
+      <c r="B25" s="2"/>
+      <c r="C25" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D25" s="5" t="s">
+        <v>30</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>